<commit_message>
updated changes to wiring diagram
</commit_message>
<xml_diff>
--- a/Documentation/wiring table.xlsx
+++ b/Documentation/wiring table.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jamcgrat\Documents\GitHub\chamberozonecontrol\Documentation\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\azale\soyface\chamberozonecontrol\Documentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{014F766E-738F-421C-A646-9A47461574B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E948B363-7162-472B-8DCD-473CEE4941E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-96" yWindow="0" windowWidth="11532" windowHeight="12336" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="182" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="192" uniqueCount="71">
   <si>
     <t>device pin</t>
   </si>
@@ -226,6 +226,18 @@
   </si>
   <si>
     <t>1-10V control (+)</t>
+  </si>
+  <si>
+    <t>male extension cord</t>
+  </si>
+  <si>
+    <t>neutral 120 V</t>
+  </si>
+  <si>
+    <t>female extension cord</t>
+  </si>
+  <si>
+    <t>ground 120 V</t>
   </si>
 </sst>
 </file>
@@ -544,19 +556,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F49"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:F51"/>
+  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="13.90625" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.81640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="26.1796875" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="14.36328125" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.08984375" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="64" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="16384" width="8.7265625" style="1"/>
+    <col min="1" max="1" width="17.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.21875" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="63.77734375" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="16384" width="8.77734375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>49</v>
       </c>
@@ -573,7 +585,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>50</v>
       </c>
@@ -581,7 +593,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>50</v>
       </c>
@@ -589,7 +601,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
         <v>50</v>
       </c>
@@ -606,7 +618,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
         <v>50</v>
       </c>
@@ -614,7 +626,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
         <v>50</v>
       </c>
@@ -631,7 +643,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
         <v>50</v>
       </c>
@@ -639,7 +651,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
         <v>50</v>
       </c>
@@ -647,7 +659,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
         <v>50</v>
       </c>
@@ -664,7 +676,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
         <v>50</v>
       </c>
@@ -681,7 +693,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
         <v>50</v>
       </c>
@@ -689,7 +701,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
         <v>50</v>
       </c>
@@ -703,7 +715,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
         <v>50</v>
       </c>
@@ -717,7 +729,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A14" s="1" t="s">
         <v>50</v>
       </c>
@@ -734,7 +746,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="s">
         <v>50</v>
       </c>
@@ -742,7 +754,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
         <v>50</v>
       </c>
@@ -750,7 +762,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A17" s="1" t="s">
         <v>50</v>
       </c>
@@ -758,7 +770,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A18" s="1" t="s">
         <v>50</v>
       </c>
@@ -775,7 +787,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A19" s="1" t="s">
         <v>50</v>
       </c>
@@ -792,7 +804,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A20" s="1" t="s">
         <v>50</v>
       </c>
@@ -800,7 +812,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A21" s="1" t="s">
         <v>50</v>
       </c>
@@ -808,7 +820,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A22" s="1" t="s">
         <v>50</v>
       </c>
@@ -816,7 +828,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A23" s="1" t="s">
         <v>50</v>
       </c>
@@ -836,7 +848,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A24" s="1" t="s">
         <v>50</v>
       </c>
@@ -856,7 +868,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A25" s="1" t="s">
         <v>50</v>
       </c>
@@ -876,7 +888,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A26" s="1" t="s">
         <v>50</v>
       </c>
@@ -896,7 +908,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A27" s="1" t="s">
         <v>50</v>
       </c>
@@ -916,7 +928,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A28" s="1" t="s">
         <v>50</v>
       </c>
@@ -936,7 +948,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A29" s="1" t="s">
         <v>50</v>
       </c>
@@ -956,7 +968,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A30" s="1" t="s">
         <v>50</v>
       </c>
@@ -964,7 +976,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A31" s="1" t="s">
         <v>50</v>
       </c>
@@ -972,7 +984,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A32" s="1" t="s">
         <v>50</v>
       </c>
@@ -980,7 +992,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A33" s="1" t="s">
         <v>50</v>
       </c>
@@ -997,7 +1009,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A34" s="1" t="s">
         <v>50</v>
       </c>
@@ -1011,7 +1023,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A35" s="1" t="s">
         <v>50</v>
       </c>
@@ -1019,7 +1031,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A36" s="1" t="s">
         <v>50</v>
       </c>
@@ -1036,7 +1048,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A37" s="1" t="s">
         <v>50</v>
       </c>
@@ -1044,7 +1056,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A38" s="1" t="s">
         <v>50</v>
       </c>
@@ -1052,7 +1064,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A39" s="1" t="s">
         <v>22</v>
       </c>
@@ -1072,7 +1084,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A40" s="1" t="s">
         <v>22</v>
       </c>
@@ -1092,7 +1104,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A41" s="1" t="s">
         <v>22</v>
       </c>
@@ -1109,7 +1121,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A42" s="1" t="s">
         <v>22</v>
       </c>
@@ -1126,7 +1138,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A43" s="1" t="s">
         <v>5</v>
       </c>
@@ -1143,12 +1155,12 @@
         <v>19</v>
       </c>
     </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A44" s="1" t="s">
         <v>5</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C44" s="1" t="s">
         <v>62</v>
@@ -1160,12 +1172,12 @@
         <v>38</v>
       </c>
     </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A45" s="1" t="s">
         <v>5</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C45" s="1" t="s">
         <v>20</v>
@@ -1177,7 +1189,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A46" s="1" t="s">
         <v>20</v>
       </c>
@@ -1194,7 +1206,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A47" s="1" t="s">
         <v>20</v>
       </c>
@@ -1214,7 +1226,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A48" s="1" t="s">
         <v>8</v>
       </c>
@@ -1231,7 +1243,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A49" s="1" t="s">
         <v>8</v>
       </c>
@@ -1246,6 +1258,40 @@
       </c>
       <c r="E49" s="1" t="s">
         <v>18</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A50" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="B50" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="C50" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="D50" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="E50" s="1" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A51" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="B51" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="C51" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="D51" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="E51" s="1" t="s">
+        <v>14</v>
       </c>
     </row>
   </sheetData>

</xml_diff>